<commit_message>
created pdf generation function
</commit_message>
<xml_diff>
--- a/templates/bingo_template.xlsx
+++ b/templates/bingo_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joelh\MusicBingo\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E776EDF1-3F72-412A-986B-2748404E23B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B85B875B-A69E-45A3-A55F-7E4B68BD0299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C07BCF10-7065-4E84-9808-49A87BD3B514}"/>
   </bookViews>
@@ -85,7 +85,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -108,19 +108,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -447,76 +459,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="33" customHeight="1">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="A1" s="3"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
     </row>
     <row r="3" spans="1:5" ht="125.1" customHeight="1">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:5" ht="125.1" customHeight="1">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:5" ht="125.1" customHeight="1">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:5" ht="125.1" customHeight="1">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:5" ht="125.1" customHeight="1">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-    </row>
-    <row r="9" spans="1:5" ht="28.5" customHeight="1">
-      <c r="A9" s="3" t="s">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:5" ht="130.5" customHeight="1">
+      <c r="A8" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" spans="1:5" ht="28.5" customHeight="1">
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
     </row>
     <row r="10" spans="1:5" ht="15" customHeight="1">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+    </row>
+    <row r="11" spans="1:5" ht="15" customHeight="1">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A9:E11"/>
+    <mergeCell ref="A8:E8"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="95" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="1.5125" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="88" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>